<commit_message>
Actualizar estado de tareas T24 y T25 en el planeamiento del Sprint 1
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/Planeamiento_Sprint1_BusTracka_1.xlsx
+++ b/planning/Planeamiento_Sprint1_BusTracka_1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/73e34dad07cdacf0/Documentos/Desktop/Ulima/Cursos/26-2/Soft 2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/73e34dad07cdacf0/Documentos/Desktop/Ulima/Cursos/26-2/Soft 2/Bustracka-Frontend-Backend-main/Bustracka-Frontend-Backend-main/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{7B801E2D-2B9C-4600-96B1-AEE6BF2E81CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8FA824AE-E414-4D7F-9EDD-D573650B61EC}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{7B801E2D-2B9C-4600-96B1-AEE6BF2E81CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{632A497C-3139-415B-BFC0-178797CEE4FA}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -977,6 +977,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -3579,7 +3583,7 @@
         <v>2</v>
       </c>
       <c r="H39" s="18" t="s">
-        <v>140</v>
+        <v>70</v>
       </c>
       <c r="I39" s="14"/>
     </row>
@@ -3606,7 +3610,7 @@
         <v>6</v>
       </c>
       <c r="H40" s="18" t="s">
-        <v>51</v>
+        <v>140</v>
       </c>
       <c r="I40" s="14"/>
     </row>

</xml_diff>